<commit_message>
Align exclusion rule (R9) with the real form's notes and add MMF test case
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PHBSGoPagpJxXxDesxZAAH
</commit_message>
<xml_diff>
--- a/vibe-coding-prep/dummy_data/answer/당사양식_정답.xlsx
+++ b/vibe-coding-prep/dummy_data/answer/당사양식_정답.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>구조화기업 아님(상장주식)</t>
+          <t>제외 대상(코스닥주식)</t>
         </is>
       </c>
     </row>
@@ -1091,32 +1091,32 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FVPL-PEF(NT)</t>
+          <t>FVPL-MMF(NT)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>감마 세컨더리 PEF 3호</t>
+          <t>알파 단기채 MMF 1호</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>KRZZ00000102</t>
+          <t>KRZZ00000110</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>감마파트너스</t>
+          <t>가상증권(주)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>대체-투자금융-PEF</t>
+          <t>단기금융</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>PEF</t>
+          <t>MMF</t>
         </is>
       </c>
       <c r="I11" s="1" t="n">
@@ -1130,15 +1130,84 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
+          <t>MMF</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>제외</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>투자금융팀</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>제외 대상(MMF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>일반계정</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>FVPL-PEF(NT)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>감마 세컨더리 PEF 3호</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>KRZZ00000102</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>감마파트너스</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>대체-투자금융-PEF</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>PEF</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="n">
+        <v>44287</v>
+      </c>
+      <c r="J12" s="1" t="n">
+        <v>47880</v>
+      </c>
+      <c r="K12" t="n">
+        <v>23800000000</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
           <t>투자펀드 및 투자신탁</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>투자금융팀</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>보고서 미수령</t>
         </is>

</xml_diff>

<commit_message>
Narrow PoC scope to total assets only; other figures are pivoted internally
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PHBSGoPagpJxXxDesxZAAH
</commit_message>
<xml_diff>
--- a/vibe-coding-prep/dummy_data/answer/당사양식_정답.xlsx
+++ b/vibe-coding-prep/dummy_data/answer/당사양식_정답.xlsx
@@ -935,9 +935,6 @@
       <c r="M8" t="n">
         <v>25992600000</v>
       </c>
-      <c r="N8" t="n">
-        <v>800000000</v>
-      </c>
       <c r="O8" t="inlineStr">
         <is>
           <t>투자금융팀</t>
@@ -1001,9 +998,6 @@
       <c r="M9" t="n">
         <v>45201100000</v>
       </c>
-      <c r="N9" t="n">
-        <v>2600000000</v>
-      </c>
       <c r="O9" t="inlineStr">
         <is>
           <t>투자금융팀</t>

</xml_diff>